<commit_message>
Update rename and recode CW XLSX
</commit_message>
<xml_diff>
--- a/Resources/Crosswalks/all_rename_variables.xlsx
+++ b/Resources/Crosswalks/all_rename_variables.xlsx
@@ -16084,7 +16084,7 @@
       </c>
       <c r="C774" t="inlineStr">
         <is>
-          <t>record_axis_code_10</t>
+          <t>record_axis_code_2</t>
         </is>
       </c>
       <c r="D774" t="b">
@@ -16104,7 +16104,7 @@
       </c>
       <c r="C775" t="inlineStr">
         <is>
-          <t>record_axis_code_11</t>
+          <t>record_axis_code_3</t>
         </is>
       </c>
       <c r="D775" t="b">
@@ -16124,7 +16124,7 @@
       </c>
       <c r="C776" t="inlineStr">
         <is>
-          <t>record_axis_code_12</t>
+          <t>record_axis_code_4</t>
         </is>
       </c>
       <c r="D776" t="b">
@@ -16144,7 +16144,7 @@
       </c>
       <c r="C777" t="inlineStr">
         <is>
-          <t>record_axis_code_13</t>
+          <t>record_axis_code_5</t>
         </is>
       </c>
       <c r="D777" t="b">
@@ -16164,7 +16164,7 @@
       </c>
       <c r="C778" t="inlineStr">
         <is>
-          <t>record_axis_code_14</t>
+          <t>record_axis_code_6</t>
         </is>
       </c>
       <c r="D778" t="b">
@@ -16184,7 +16184,7 @@
       </c>
       <c r="C779" t="inlineStr">
         <is>
-          <t>record_axis_code_15</t>
+          <t>record_axis_code_7</t>
         </is>
       </c>
       <c r="D779" t="b">
@@ -16204,7 +16204,7 @@
       </c>
       <c r="C780" t="inlineStr">
         <is>
-          <t>record_axis_code_16</t>
+          <t>record_axis_code_8</t>
         </is>
       </c>
       <c r="D780" t="b">
@@ -16224,7 +16224,7 @@
       </c>
       <c r="C781" t="inlineStr">
         <is>
-          <t>record_axis_code_17</t>
+          <t>record_axis_code_9</t>
         </is>
       </c>
       <c r="D781" t="b">
@@ -16244,7 +16244,7 @@
       </c>
       <c r="C782" t="inlineStr">
         <is>
-          <t>record_axis_code_18</t>
+          <t>record_axis_code_10</t>
         </is>
       </c>
       <c r="D782" t="b">
@@ -16264,7 +16264,7 @@
       </c>
       <c r="C783" t="inlineStr">
         <is>
-          <t>record_axis_code_19</t>
+          <t>record_axis_code_11</t>
         </is>
       </c>
       <c r="D783" t="b">
@@ -16284,7 +16284,7 @@
       </c>
       <c r="C784" t="inlineStr">
         <is>
-          <t>record_axis_code_2</t>
+          <t>record_axis_code_12</t>
         </is>
       </c>
       <c r="D784" t="b">
@@ -16304,7 +16304,7 @@
       </c>
       <c r="C785" t="inlineStr">
         <is>
-          <t>record_axis_code_20</t>
+          <t>record_axis_code_13</t>
         </is>
       </c>
       <c r="D785" t="b">
@@ -16324,7 +16324,7 @@
       </c>
       <c r="C786" t="inlineStr">
         <is>
-          <t>record_axis_code_3</t>
+          <t>record_axis_code_14</t>
         </is>
       </c>
       <c r="D786" t="b">
@@ -16344,7 +16344,7 @@
       </c>
       <c r="C787" t="inlineStr">
         <is>
-          <t>record_axis_code_4</t>
+          <t>record_axis_code_15</t>
         </is>
       </c>
       <c r="D787" t="b">
@@ -16364,7 +16364,7 @@
       </c>
       <c r="C788" t="inlineStr">
         <is>
-          <t>record_axis_code_5</t>
+          <t>record_axis_code_16</t>
         </is>
       </c>
       <c r="D788" t="b">
@@ -16384,7 +16384,7 @@
       </c>
       <c r="C789" t="inlineStr">
         <is>
-          <t>record_axis_code_6</t>
+          <t>record_axis_code_17</t>
         </is>
       </c>
       <c r="D789" t="b">
@@ -16404,7 +16404,7 @@
       </c>
       <c r="C790" t="inlineStr">
         <is>
-          <t>record_axis_code_7</t>
+          <t>record_axis_code_18</t>
         </is>
       </c>
       <c r="D790" t="b">
@@ -16424,7 +16424,7 @@
       </c>
       <c r="C791" t="inlineStr">
         <is>
-          <t>record_axis_code_8</t>
+          <t>record_axis_code_19</t>
         </is>
       </c>
       <c r="D791" t="b">
@@ -16444,7 +16444,7 @@
       </c>
       <c r="C792" t="inlineStr">
         <is>
-          <t>record_axis_code_9</t>
+          <t>record_axis_code_20</t>
         </is>
       </c>
       <c r="D792" t="b">
@@ -18124,7 +18124,7 @@
       </c>
       <c r="C875" t="inlineStr">
         <is>
-          <t>record_axis_code_10</t>
+          <t>record_axis_code_2</t>
         </is>
       </c>
       <c r="D875" t="b">
@@ -18144,7 +18144,7 @@
       </c>
       <c r="C876" t="inlineStr">
         <is>
-          <t>record_axis_code_11</t>
+          <t>record_axis_code_3</t>
         </is>
       </c>
       <c r="D876" t="b">
@@ -18164,7 +18164,7 @@
       </c>
       <c r="C877" t="inlineStr">
         <is>
-          <t>record_axis_code_12</t>
+          <t>record_axis_code_4</t>
         </is>
       </c>
       <c r="D877" t="b">
@@ -18184,7 +18184,7 @@
       </c>
       <c r="C878" t="inlineStr">
         <is>
-          <t>record_axis_code_13</t>
+          <t>record_axis_code_5</t>
         </is>
       </c>
       <c r="D878" t="b">
@@ -18204,7 +18204,7 @@
       </c>
       <c r="C879" t="inlineStr">
         <is>
-          <t>record_axis_code_14</t>
+          <t>record_axis_code_6</t>
         </is>
       </c>
       <c r="D879" t="b">
@@ -18224,7 +18224,7 @@
       </c>
       <c r="C880" t="inlineStr">
         <is>
-          <t>record_axis_code_15</t>
+          <t>record_axis_code_7</t>
         </is>
       </c>
       <c r="D880" t="b">
@@ -18244,7 +18244,7 @@
       </c>
       <c r="C881" t="inlineStr">
         <is>
-          <t>record_axis_code_16</t>
+          <t>record_axis_code_8</t>
         </is>
       </c>
       <c r="D881" t="b">
@@ -18264,7 +18264,7 @@
       </c>
       <c r="C882" t="inlineStr">
         <is>
-          <t>record_axis_code_17</t>
+          <t>record_axis_code_9</t>
         </is>
       </c>
       <c r="D882" t="b">
@@ -18284,7 +18284,7 @@
       </c>
       <c r="C883" t="inlineStr">
         <is>
-          <t>record_axis_code_18</t>
+          <t>record_axis_code_10</t>
         </is>
       </c>
       <c r="D883" t="b">
@@ -18304,7 +18304,7 @@
       </c>
       <c r="C884" t="inlineStr">
         <is>
-          <t>record_axis_code_19</t>
+          <t>record_axis_code_11</t>
         </is>
       </c>
       <c r="D884" t="b">
@@ -18324,7 +18324,7 @@
       </c>
       <c r="C885" t="inlineStr">
         <is>
-          <t>record_axis_code_2</t>
+          <t>record_axis_code_12</t>
         </is>
       </c>
       <c r="D885" t="b">
@@ -18344,7 +18344,7 @@
       </c>
       <c r="C886" t="inlineStr">
         <is>
-          <t>record_axis_code_20</t>
+          <t>record_axis_code_13</t>
         </is>
       </c>
       <c r="D886" t="b">
@@ -18364,7 +18364,7 @@
       </c>
       <c r="C887" t="inlineStr">
         <is>
-          <t>record_axis_code_3</t>
+          <t>record_axis_code_14</t>
         </is>
       </c>
       <c r="D887" t="b">
@@ -18384,7 +18384,7 @@
       </c>
       <c r="C888" t="inlineStr">
         <is>
-          <t>record_axis_code_4</t>
+          <t>record_axis_code_15</t>
         </is>
       </c>
       <c r="D888" t="b">
@@ -18404,7 +18404,7 @@
       </c>
       <c r="C889" t="inlineStr">
         <is>
-          <t>record_axis_code_5</t>
+          <t>record_axis_code_16</t>
         </is>
       </c>
       <c r="D889" t="b">
@@ -18424,7 +18424,7 @@
       </c>
       <c r="C890" t="inlineStr">
         <is>
-          <t>record_axis_code_6</t>
+          <t>record_axis_code_17</t>
         </is>
       </c>
       <c r="D890" t="b">
@@ -18444,7 +18444,7 @@
       </c>
       <c r="C891" t="inlineStr">
         <is>
-          <t>record_axis_code_7</t>
+          <t>record_axis_code_18</t>
         </is>
       </c>
       <c r="D891" t="b">
@@ -18464,7 +18464,7 @@
       </c>
       <c r="C892" t="inlineStr">
         <is>
-          <t>record_axis_code_8</t>
+          <t>record_axis_code_19</t>
         </is>
       </c>
       <c r="D892" t="b">
@@ -18484,7 +18484,7 @@
       </c>
       <c r="C893" t="inlineStr">
         <is>
-          <t>record_axis_code_9</t>
+          <t>record_axis_code_20</t>
         </is>
       </c>
       <c r="D893" t="b">
@@ -20164,7 +20164,7 @@
       </c>
       <c r="C976" t="inlineStr">
         <is>
-          <t>record_axis_code_10</t>
+          <t>record_axis_code_2</t>
         </is>
       </c>
       <c r="D976" t="b">
@@ -20184,7 +20184,7 @@
       </c>
       <c r="C977" t="inlineStr">
         <is>
-          <t>record_axis_code_11</t>
+          <t>record_axis_code_3</t>
         </is>
       </c>
       <c r="D977" t="b">
@@ -20204,7 +20204,7 @@
       </c>
       <c r="C978" t="inlineStr">
         <is>
-          <t>record_axis_code_12</t>
+          <t>record_axis_code_4</t>
         </is>
       </c>
       <c r="D978" t="b">
@@ -20224,7 +20224,7 @@
       </c>
       <c r="C979" t="inlineStr">
         <is>
-          <t>record_axis_code_13</t>
+          <t>record_axis_code_5</t>
         </is>
       </c>
       <c r="D979" t="b">
@@ -20244,7 +20244,7 @@
       </c>
       <c r="C980" t="inlineStr">
         <is>
-          <t>record_axis_code_14</t>
+          <t>record_axis_code_6</t>
         </is>
       </c>
       <c r="D980" t="b">
@@ -20264,7 +20264,7 @@
       </c>
       <c r="C981" t="inlineStr">
         <is>
-          <t>record_axis_code_15</t>
+          <t>record_axis_code_7</t>
         </is>
       </c>
       <c r="D981" t="b">
@@ -20284,7 +20284,7 @@
       </c>
       <c r="C982" t="inlineStr">
         <is>
-          <t>record_axis_code_16</t>
+          <t>record_axis_code_8</t>
         </is>
       </c>
       <c r="D982" t="b">
@@ -20304,7 +20304,7 @@
       </c>
       <c r="C983" t="inlineStr">
         <is>
-          <t>record_axis_code_17</t>
+          <t>record_axis_code_9</t>
         </is>
       </c>
       <c r="D983" t="b">
@@ -20324,7 +20324,7 @@
       </c>
       <c r="C984" t="inlineStr">
         <is>
-          <t>record_axis_code_18</t>
+          <t>record_axis_code_10</t>
         </is>
       </c>
       <c r="D984" t="b">
@@ -20344,7 +20344,7 @@
       </c>
       <c r="C985" t="inlineStr">
         <is>
-          <t>record_axis_code_19</t>
+          <t>record_axis_code_11</t>
         </is>
       </c>
       <c r="D985" t="b">
@@ -20364,7 +20364,7 @@
       </c>
       <c r="C986" t="inlineStr">
         <is>
-          <t>record_axis_code_2</t>
+          <t>record_axis_code_12</t>
         </is>
       </c>
       <c r="D986" t="b">
@@ -20384,7 +20384,7 @@
       </c>
       <c r="C987" t="inlineStr">
         <is>
-          <t>record_axis_code_20</t>
+          <t>record_axis_code_13</t>
         </is>
       </c>
       <c r="D987" t="b">
@@ -20404,7 +20404,7 @@
       </c>
       <c r="C988" t="inlineStr">
         <is>
-          <t>record_axis_code_3</t>
+          <t>record_axis_code_14</t>
         </is>
       </c>
       <c r="D988" t="b">
@@ -20424,7 +20424,7 @@
       </c>
       <c r="C989" t="inlineStr">
         <is>
-          <t>record_axis_code_4</t>
+          <t>record_axis_code_15</t>
         </is>
       </c>
       <c r="D989" t="b">
@@ -20444,7 +20444,7 @@
       </c>
       <c r="C990" t="inlineStr">
         <is>
-          <t>record_axis_code_5</t>
+          <t>record_axis_code_16</t>
         </is>
       </c>
       <c r="D990" t="b">
@@ -20464,7 +20464,7 @@
       </c>
       <c r="C991" t="inlineStr">
         <is>
-          <t>record_axis_code_6</t>
+          <t>record_axis_code_17</t>
         </is>
       </c>
       <c r="D991" t="b">
@@ -20484,7 +20484,7 @@
       </c>
       <c r="C992" t="inlineStr">
         <is>
-          <t>record_axis_code_7</t>
+          <t>record_axis_code_18</t>
         </is>
       </c>
       <c r="D992" t="b">
@@ -20504,7 +20504,7 @@
       </c>
       <c r="C993" t="inlineStr">
         <is>
-          <t>record_axis_code_8</t>
+          <t>record_axis_code_19</t>
         </is>
       </c>
       <c r="D993" t="b">
@@ -20524,7 +20524,7 @@
       </c>
       <c r="C994" t="inlineStr">
         <is>
-          <t>record_axis_code_9</t>
+          <t>record_axis_code_20</t>
         </is>
       </c>
       <c r="D994" t="b">
@@ -22204,7 +22204,7 @@
       </c>
       <c r="C1077" t="inlineStr">
         <is>
-          <t>record_axis_code_10</t>
+          <t>record_axis_code_2</t>
         </is>
       </c>
       <c r="D1077" t="b">
@@ -22224,7 +22224,7 @@
       </c>
       <c r="C1078" t="inlineStr">
         <is>
-          <t>record_axis_code_11</t>
+          <t>record_axis_code_3</t>
         </is>
       </c>
       <c r="D1078" t="b">
@@ -22244,7 +22244,7 @@
       </c>
       <c r="C1079" t="inlineStr">
         <is>
-          <t>record_axis_code_12</t>
+          <t>record_axis_code_4</t>
         </is>
       </c>
       <c r="D1079" t="b">
@@ -22264,7 +22264,7 @@
       </c>
       <c r="C1080" t="inlineStr">
         <is>
-          <t>record_axis_code_13</t>
+          <t>record_axis_code_5</t>
         </is>
       </c>
       <c r="D1080" t="b">
@@ -22284,7 +22284,7 @@
       </c>
       <c r="C1081" t="inlineStr">
         <is>
-          <t>record_axis_code_14</t>
+          <t>record_axis_code_6</t>
         </is>
       </c>
       <c r="D1081" t="b">
@@ -22304,7 +22304,7 @@
       </c>
       <c r="C1082" t="inlineStr">
         <is>
-          <t>record_axis_code_15</t>
+          <t>record_axis_code_7</t>
         </is>
       </c>
       <c r="D1082" t="b">
@@ -22324,7 +22324,7 @@
       </c>
       <c r="C1083" t="inlineStr">
         <is>
-          <t>record_axis_code_16</t>
+          <t>record_axis_code_8</t>
         </is>
       </c>
       <c r="D1083" t="b">
@@ -22344,7 +22344,7 @@
       </c>
       <c r="C1084" t="inlineStr">
         <is>
-          <t>record_axis_code_17</t>
+          <t>record_axis_code_9</t>
         </is>
       </c>
       <c r="D1084" t="b">
@@ -22364,7 +22364,7 @@
       </c>
       <c r="C1085" t="inlineStr">
         <is>
-          <t>record_axis_code_18</t>
+          <t>record_axis_code_10</t>
         </is>
       </c>
       <c r="D1085" t="b">
@@ -22384,7 +22384,7 @@
       </c>
       <c r="C1086" t="inlineStr">
         <is>
-          <t>record_axis_code_19</t>
+          <t>record_axis_code_11</t>
         </is>
       </c>
       <c r="D1086" t="b">
@@ -22404,7 +22404,7 @@
       </c>
       <c r="C1087" t="inlineStr">
         <is>
-          <t>record_axis_code_2</t>
+          <t>record_axis_code_12</t>
         </is>
       </c>
       <c r="D1087" t="b">
@@ -22424,7 +22424,7 @@
       </c>
       <c r="C1088" t="inlineStr">
         <is>
-          <t>record_axis_code_20</t>
+          <t>record_axis_code_13</t>
         </is>
       </c>
       <c r="D1088" t="b">
@@ -22444,7 +22444,7 @@
       </c>
       <c r="C1089" t="inlineStr">
         <is>
-          <t>record_axis_code_3</t>
+          <t>record_axis_code_14</t>
         </is>
       </c>
       <c r="D1089" t="b">
@@ -22464,7 +22464,7 @@
       </c>
       <c r="C1090" t="inlineStr">
         <is>
-          <t>record_axis_code_4</t>
+          <t>record_axis_code_15</t>
         </is>
       </c>
       <c r="D1090" t="b">
@@ -22484,7 +22484,7 @@
       </c>
       <c r="C1091" t="inlineStr">
         <is>
-          <t>record_axis_code_5</t>
+          <t>record_axis_code_16</t>
         </is>
       </c>
       <c r="D1091" t="b">
@@ -22504,7 +22504,7 @@
       </c>
       <c r="C1092" t="inlineStr">
         <is>
-          <t>record_axis_code_6</t>
+          <t>record_axis_code_17</t>
         </is>
       </c>
       <c r="D1092" t="b">
@@ -22524,7 +22524,7 @@
       </c>
       <c r="C1093" t="inlineStr">
         <is>
-          <t>record_axis_code_7</t>
+          <t>record_axis_code_18</t>
         </is>
       </c>
       <c r="D1093" t="b">
@@ -22544,7 +22544,7 @@
       </c>
       <c r="C1094" t="inlineStr">
         <is>
-          <t>record_axis_code_8</t>
+          <t>record_axis_code_19</t>
         </is>
       </c>
       <c r="D1094" t="b">
@@ -22564,7 +22564,7 @@
       </c>
       <c r="C1095" t="inlineStr">
         <is>
-          <t>record_axis_code_9</t>
+          <t>record_axis_code_20</t>
         </is>
       </c>
       <c r="D1095" t="b">
@@ -24244,7 +24244,7 @@
       </c>
       <c r="C1178" t="inlineStr">
         <is>
-          <t>record_axis_code_10</t>
+          <t>record_axis_code_2</t>
         </is>
       </c>
       <c r="D1178" t="b">
@@ -24264,7 +24264,7 @@
       </c>
       <c r="C1179" t="inlineStr">
         <is>
-          <t>record_axis_code_11</t>
+          <t>record_axis_code_3</t>
         </is>
       </c>
       <c r="D1179" t="b">
@@ -24284,7 +24284,7 @@
       </c>
       <c r="C1180" t="inlineStr">
         <is>
-          <t>record_axis_code_12</t>
+          <t>record_axis_code_4</t>
         </is>
       </c>
       <c r="D1180" t="b">
@@ -24304,7 +24304,7 @@
       </c>
       <c r="C1181" t="inlineStr">
         <is>
-          <t>record_axis_code_13</t>
+          <t>record_axis_code_5</t>
         </is>
       </c>
       <c r="D1181" t="b">
@@ -24324,7 +24324,7 @@
       </c>
       <c r="C1182" t="inlineStr">
         <is>
-          <t>record_axis_code_14</t>
+          <t>record_axis_code_6</t>
         </is>
       </c>
       <c r="D1182" t="b">
@@ -24344,7 +24344,7 @@
       </c>
       <c r="C1183" t="inlineStr">
         <is>
-          <t>record_axis_code_15</t>
+          <t>record_axis_code_7</t>
         </is>
       </c>
       <c r="D1183" t="b">
@@ -24364,7 +24364,7 @@
       </c>
       <c r="C1184" t="inlineStr">
         <is>
-          <t>record_axis_code_16</t>
+          <t>record_axis_code_8</t>
         </is>
       </c>
       <c r="D1184" t="b">
@@ -24384,7 +24384,7 @@
       </c>
       <c r="C1185" t="inlineStr">
         <is>
-          <t>record_axis_code_17</t>
+          <t>record_axis_code_9</t>
         </is>
       </c>
       <c r="D1185" t="b">
@@ -24404,7 +24404,7 @@
       </c>
       <c r="C1186" t="inlineStr">
         <is>
-          <t>record_axis_code_18</t>
+          <t>record_axis_code_10</t>
         </is>
       </c>
       <c r="D1186" t="b">
@@ -24424,7 +24424,7 @@
       </c>
       <c r="C1187" t="inlineStr">
         <is>
-          <t>record_axis_code_19</t>
+          <t>record_axis_code_11</t>
         </is>
       </c>
       <c r="D1187" t="b">
@@ -24444,7 +24444,7 @@
       </c>
       <c r="C1188" t="inlineStr">
         <is>
-          <t>record_axis_code_2</t>
+          <t>record_axis_code_12</t>
         </is>
       </c>
       <c r="D1188" t="b">
@@ -24464,7 +24464,7 @@
       </c>
       <c r="C1189" t="inlineStr">
         <is>
-          <t>record_axis_code_20</t>
+          <t>record_axis_code_13</t>
         </is>
       </c>
       <c r="D1189" t="b">
@@ -24484,7 +24484,7 @@
       </c>
       <c r="C1190" t="inlineStr">
         <is>
-          <t>record_axis_code_3</t>
+          <t>record_axis_code_14</t>
         </is>
       </c>
       <c r="D1190" t="b">
@@ -24504,7 +24504,7 @@
       </c>
       <c r="C1191" t="inlineStr">
         <is>
-          <t>record_axis_code_4</t>
+          <t>record_axis_code_15</t>
         </is>
       </c>
       <c r="D1191" t="b">
@@ -24524,7 +24524,7 @@
       </c>
       <c r="C1192" t="inlineStr">
         <is>
-          <t>record_axis_code_5</t>
+          <t>record_axis_code_16</t>
         </is>
       </c>
       <c r="D1192" t="b">
@@ -24544,7 +24544,7 @@
       </c>
       <c r="C1193" t="inlineStr">
         <is>
-          <t>record_axis_code_6</t>
+          <t>record_axis_code_17</t>
         </is>
       </c>
       <c r="D1193" t="b">
@@ -24564,7 +24564,7 @@
       </c>
       <c r="C1194" t="inlineStr">
         <is>
-          <t>record_axis_code_7</t>
+          <t>record_axis_code_18</t>
         </is>
       </c>
       <c r="D1194" t="b">
@@ -24584,7 +24584,7 @@
       </c>
       <c r="C1195" t="inlineStr">
         <is>
-          <t>record_axis_code_8</t>
+          <t>record_axis_code_19</t>
         </is>
       </c>
       <c r="D1195" t="b">
@@ -24604,7 +24604,7 @@
       </c>
       <c r="C1196" t="inlineStr">
         <is>
-          <t>record_axis_code_9</t>
+          <t>record_axis_code_20</t>
         </is>
       </c>
       <c r="D1196" t="b">
@@ -26304,7 +26304,7 @@
       </c>
       <c r="C1279" t="inlineStr">
         <is>
-          <t>record_axis_code_10</t>
+          <t>record_axis_code_2</t>
         </is>
       </c>
       <c r="D1279" t="b">
@@ -26324,7 +26324,7 @@
       </c>
       <c r="C1280" t="inlineStr">
         <is>
-          <t>record_axis_code_11</t>
+          <t>record_axis_code_3</t>
         </is>
       </c>
       <c r="D1280" t="b">
@@ -26344,7 +26344,7 @@
       </c>
       <c r="C1281" t="inlineStr">
         <is>
-          <t>record_axis_code_12</t>
+          <t>record_axis_code_4</t>
         </is>
       </c>
       <c r="D1281" t="b">
@@ -26364,7 +26364,7 @@
       </c>
       <c r="C1282" t="inlineStr">
         <is>
-          <t>record_axis_code_13</t>
+          <t>record_axis_code_5</t>
         </is>
       </c>
       <c r="D1282" t="b">
@@ -26384,7 +26384,7 @@
       </c>
       <c r="C1283" t="inlineStr">
         <is>
-          <t>record_axis_code_14</t>
+          <t>record_axis_code_6</t>
         </is>
       </c>
       <c r="D1283" t="b">
@@ -26404,7 +26404,7 @@
       </c>
       <c r="C1284" t="inlineStr">
         <is>
-          <t>record_axis_code_15</t>
+          <t>record_axis_code_7</t>
         </is>
       </c>
       <c r="D1284" t="b">
@@ -26424,7 +26424,7 @@
       </c>
       <c r="C1285" t="inlineStr">
         <is>
-          <t>record_axis_code_16</t>
+          <t>record_axis_code_8</t>
         </is>
       </c>
       <c r="D1285" t="b">
@@ -26444,7 +26444,7 @@
       </c>
       <c r="C1286" t="inlineStr">
         <is>
-          <t>record_axis_code_17</t>
+          <t>record_axis_code_9</t>
         </is>
       </c>
       <c r="D1286" t="b">
@@ -26464,7 +26464,7 @@
       </c>
       <c r="C1287" t="inlineStr">
         <is>
-          <t>record_axis_code_18</t>
+          <t>record_axis_code_10</t>
         </is>
       </c>
       <c r="D1287" t="b">
@@ -26484,7 +26484,7 @@
       </c>
       <c r="C1288" t="inlineStr">
         <is>
-          <t>record_axis_code_19</t>
+          <t>record_axis_code_11</t>
         </is>
       </c>
       <c r="D1288" t="b">
@@ -26504,7 +26504,7 @@
       </c>
       <c r="C1289" t="inlineStr">
         <is>
-          <t>record_axis_code_2</t>
+          <t>record_axis_code_12</t>
         </is>
       </c>
       <c r="D1289" t="b">
@@ -26524,7 +26524,7 @@
       </c>
       <c r="C1290" t="inlineStr">
         <is>
-          <t>record_axis_code_20</t>
+          <t>record_axis_code_13</t>
         </is>
       </c>
       <c r="D1290" t="b">
@@ -26544,7 +26544,7 @@
       </c>
       <c r="C1291" t="inlineStr">
         <is>
-          <t>record_axis_code_3</t>
+          <t>record_axis_code_14</t>
         </is>
       </c>
       <c r="D1291" t="b">
@@ -26564,7 +26564,7 @@
       </c>
       <c r="C1292" t="inlineStr">
         <is>
-          <t>record_axis_code_4</t>
+          <t>record_axis_code_15</t>
         </is>
       </c>
       <c r="D1292" t="b">
@@ -26584,7 +26584,7 @@
       </c>
       <c r="C1293" t="inlineStr">
         <is>
-          <t>record_axis_code_5</t>
+          <t>record_axis_code_16</t>
         </is>
       </c>
       <c r="D1293" t="b">
@@ -26604,7 +26604,7 @@
       </c>
       <c r="C1294" t="inlineStr">
         <is>
-          <t>record_axis_code_6</t>
+          <t>record_axis_code_17</t>
         </is>
       </c>
       <c r="D1294" t="b">
@@ -26624,7 +26624,7 @@
       </c>
       <c r="C1295" t="inlineStr">
         <is>
-          <t>record_axis_code_7</t>
+          <t>record_axis_code_18</t>
         </is>
       </c>
       <c r="D1295" t="b">
@@ -26644,7 +26644,7 @@
       </c>
       <c r="C1296" t="inlineStr">
         <is>
-          <t>record_axis_code_8</t>
+          <t>record_axis_code_19</t>
         </is>
       </c>
       <c r="D1296" t="b">
@@ -26664,7 +26664,7 @@
       </c>
       <c r="C1297" t="inlineStr">
         <is>
-          <t>record_axis_code_9</t>
+          <t>record_axis_code_20</t>
         </is>
       </c>
       <c r="D1297" t="b">
@@ -28374,7 +28374,7 @@
       </c>
       <c r="C1380" t="inlineStr">
         <is>
-          <t>record_axis_code_10</t>
+          <t>record_axis_code_2</t>
         </is>
       </c>
       <c r="D1380" t="b">
@@ -28394,7 +28394,7 @@
       </c>
       <c r="C1381" t="inlineStr">
         <is>
-          <t>record_axis_code_11</t>
+          <t>record_axis_code_3</t>
         </is>
       </c>
       <c r="D1381" t="b">
@@ -28414,7 +28414,7 @@
       </c>
       <c r="C1382" t="inlineStr">
         <is>
-          <t>record_axis_code_12</t>
+          <t>record_axis_code_4</t>
         </is>
       </c>
       <c r="D1382" t="b">
@@ -28434,7 +28434,7 @@
       </c>
       <c r="C1383" t="inlineStr">
         <is>
-          <t>record_axis_code_13</t>
+          <t>record_axis_code_5</t>
         </is>
       </c>
       <c r="D1383" t="b">
@@ -28454,7 +28454,7 @@
       </c>
       <c r="C1384" t="inlineStr">
         <is>
-          <t>record_axis_code_14</t>
+          <t>record_axis_code_6</t>
         </is>
       </c>
       <c r="D1384" t="b">
@@ -28474,7 +28474,7 @@
       </c>
       <c r="C1385" t="inlineStr">
         <is>
-          <t>record_axis_code_15</t>
+          <t>record_axis_code_7</t>
         </is>
       </c>
       <c r="D1385" t="b">
@@ -28494,7 +28494,7 @@
       </c>
       <c r="C1386" t="inlineStr">
         <is>
-          <t>record_axis_code_16</t>
+          <t>record_axis_code_8</t>
         </is>
       </c>
       <c r="D1386" t="b">
@@ -28514,7 +28514,7 @@
       </c>
       <c r="C1387" t="inlineStr">
         <is>
-          <t>record_axis_code_17</t>
+          <t>record_axis_code_9</t>
         </is>
       </c>
       <c r="D1387" t="b">
@@ -28534,7 +28534,7 @@
       </c>
       <c r="C1388" t="inlineStr">
         <is>
-          <t>record_axis_code_18</t>
+          <t>record_axis_code_10</t>
         </is>
       </c>
       <c r="D1388" t="b">
@@ -28554,7 +28554,7 @@
       </c>
       <c r="C1389" t="inlineStr">
         <is>
-          <t>record_axis_code_19</t>
+          <t>record_axis_code_11</t>
         </is>
       </c>
       <c r="D1389" t="b">
@@ -28574,7 +28574,7 @@
       </c>
       <c r="C1390" t="inlineStr">
         <is>
-          <t>record_axis_code_2</t>
+          <t>record_axis_code_12</t>
         </is>
       </c>
       <c r="D1390" t="b">
@@ -28594,7 +28594,7 @@
       </c>
       <c r="C1391" t="inlineStr">
         <is>
-          <t>record_axis_code_20</t>
+          <t>record_axis_code_13</t>
         </is>
       </c>
       <c r="D1391" t="b">
@@ -28614,7 +28614,7 @@
       </c>
       <c r="C1392" t="inlineStr">
         <is>
-          <t>record_axis_code_3</t>
+          <t>record_axis_code_14</t>
         </is>
       </c>
       <c r="D1392" t="b">
@@ -28634,7 +28634,7 @@
       </c>
       <c r="C1393" t="inlineStr">
         <is>
-          <t>record_axis_code_4</t>
+          <t>record_axis_code_15</t>
         </is>
       </c>
       <c r="D1393" t="b">
@@ -28654,7 +28654,7 @@
       </c>
       <c r="C1394" t="inlineStr">
         <is>
-          <t>record_axis_code_5</t>
+          <t>record_axis_code_16</t>
         </is>
       </c>
       <c r="D1394" t="b">
@@ -28674,7 +28674,7 @@
       </c>
       <c r="C1395" t="inlineStr">
         <is>
-          <t>record_axis_code_6</t>
+          <t>record_axis_code_17</t>
         </is>
       </c>
       <c r="D1395" t="b">
@@ -28694,7 +28694,7 @@
       </c>
       <c r="C1396" t="inlineStr">
         <is>
-          <t>record_axis_code_7</t>
+          <t>record_axis_code_18</t>
         </is>
       </c>
       <c r="D1396" t="b">
@@ -28714,7 +28714,7 @@
       </c>
       <c r="C1397" t="inlineStr">
         <is>
-          <t>record_axis_code_8</t>
+          <t>record_axis_code_19</t>
         </is>
       </c>
       <c r="D1397" t="b">
@@ -28734,7 +28734,7 @@
       </c>
       <c r="C1398" t="inlineStr">
         <is>
-          <t>record_axis_code_9</t>
+          <t>record_axis_code_20</t>
         </is>
       </c>
       <c r="D1398" t="b">
@@ -30444,7 +30444,7 @@
       </c>
       <c r="C1481" t="inlineStr">
         <is>
-          <t>record_axis_code_10</t>
+          <t>record_axis_code_2</t>
         </is>
       </c>
       <c r="D1481" t="b">
@@ -30464,7 +30464,7 @@
       </c>
       <c r="C1482" t="inlineStr">
         <is>
-          <t>record_axis_code_11</t>
+          <t>record_axis_code_3</t>
         </is>
       </c>
       <c r="D1482" t="b">
@@ -30484,7 +30484,7 @@
       </c>
       <c r="C1483" t="inlineStr">
         <is>
-          <t>record_axis_code_12</t>
+          <t>record_axis_code_4</t>
         </is>
       </c>
       <c r="D1483" t="b">
@@ -30504,7 +30504,7 @@
       </c>
       <c r="C1484" t="inlineStr">
         <is>
-          <t>record_axis_code_13</t>
+          <t>record_axis_code_5</t>
         </is>
       </c>
       <c r="D1484" t="b">
@@ -30524,7 +30524,7 @@
       </c>
       <c r="C1485" t="inlineStr">
         <is>
-          <t>record_axis_code_14</t>
+          <t>record_axis_code_6</t>
         </is>
       </c>
       <c r="D1485" t="b">
@@ -30544,7 +30544,7 @@
       </c>
       <c r="C1486" t="inlineStr">
         <is>
-          <t>record_axis_code_15</t>
+          <t>record_axis_code_7</t>
         </is>
       </c>
       <c r="D1486" t="b">
@@ -30564,7 +30564,7 @@
       </c>
       <c r="C1487" t="inlineStr">
         <is>
-          <t>record_axis_code_16</t>
+          <t>record_axis_code_8</t>
         </is>
       </c>
       <c r="D1487" t="b">
@@ -30584,7 +30584,7 @@
       </c>
       <c r="C1488" t="inlineStr">
         <is>
-          <t>record_axis_code_17</t>
+          <t>record_axis_code_9</t>
         </is>
       </c>
       <c r="D1488" t="b">
@@ -30604,7 +30604,7 @@
       </c>
       <c r="C1489" t="inlineStr">
         <is>
-          <t>record_axis_code_18</t>
+          <t>record_axis_code_10</t>
         </is>
       </c>
       <c r="D1489" t="b">
@@ -30624,7 +30624,7 @@
       </c>
       <c r="C1490" t="inlineStr">
         <is>
-          <t>record_axis_code_19</t>
+          <t>record_axis_code_11</t>
         </is>
       </c>
       <c r="D1490" t="b">
@@ -30644,7 +30644,7 @@
       </c>
       <c r="C1491" t="inlineStr">
         <is>
-          <t>record_axis_code_2</t>
+          <t>record_axis_code_12</t>
         </is>
       </c>
       <c r="D1491" t="b">
@@ -30664,7 +30664,7 @@
       </c>
       <c r="C1492" t="inlineStr">
         <is>
-          <t>record_axis_code_20</t>
+          <t>record_axis_code_13</t>
         </is>
       </c>
       <c r="D1492" t="b">
@@ -30684,7 +30684,7 @@
       </c>
       <c r="C1493" t="inlineStr">
         <is>
-          <t>record_axis_code_3</t>
+          <t>record_axis_code_14</t>
         </is>
       </c>
       <c r="D1493" t="b">
@@ -30704,7 +30704,7 @@
       </c>
       <c r="C1494" t="inlineStr">
         <is>
-          <t>record_axis_code_4</t>
+          <t>record_axis_code_15</t>
         </is>
       </c>
       <c r="D1494" t="b">
@@ -30724,7 +30724,7 @@
       </c>
       <c r="C1495" t="inlineStr">
         <is>
-          <t>record_axis_code_5</t>
+          <t>record_axis_code_16</t>
         </is>
       </c>
       <c r="D1495" t="b">
@@ -30744,7 +30744,7 @@
       </c>
       <c r="C1496" t="inlineStr">
         <is>
-          <t>record_axis_code_6</t>
+          <t>record_axis_code_17</t>
         </is>
       </c>
       <c r="D1496" t="b">
@@ -30764,7 +30764,7 @@
       </c>
       <c r="C1497" t="inlineStr">
         <is>
-          <t>record_axis_code_7</t>
+          <t>record_axis_code_18</t>
         </is>
       </c>
       <c r="D1497" t="b">
@@ -30784,7 +30784,7 @@
       </c>
       <c r="C1498" t="inlineStr">
         <is>
-          <t>record_axis_code_8</t>
+          <t>record_axis_code_19</t>
         </is>
       </c>
       <c r="D1498" t="b">
@@ -30804,7 +30804,7 @@
       </c>
       <c r="C1499" t="inlineStr">
         <is>
-          <t>record_axis_code_9</t>
+          <t>record_axis_code_20</t>
         </is>
       </c>
       <c r="D1499" t="b">

</xml_diff>